<commit_message>
Updated DEU_grids_kan model - 2025-12-05 17:05
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_DEU_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4C4C18F-6948-4D38-8CB7-CCE22DD0E55C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5976EE16-FF85-4D1E-A193-52AE3E51449E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="12683" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="56" r:id="rId1"/>
@@ -35646,7 +35646,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE00BE76-82D4-471D-B927-FCA81A392AE0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1763BE15-3A80-4491-8ABA-EC97C9553B00}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -46332,7 +46332,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E3A877A-0C5F-4025-B994-B662EE5A4F62}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87F8BDF4-3DA2-4925-ADAD-4095FEB4727F}">
   <dimension ref="B9:L546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DEU_grids_kan model - 2025-12-05 19:10
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_DEU_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5976EE16-FF85-4D1E-A193-52AE3E51449E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B52BA2B0-64E5-481C-8786-E3F5C7A14579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="12683" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="56" r:id="rId1"/>
@@ -35646,7 +35646,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1763BE15-3A80-4491-8ABA-EC97C9553B00}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBE54553-334A-4352-BAF1-F63A1A0048A9}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -46332,7 +46332,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87F8BDF4-3DA2-4925-ADAD-4095FEB4727F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07A2BB65-16D3-4A47-B016-80C82AC7F476}">
   <dimension ref="B9:L546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>